<commit_message>
Add a new environment to test the model
</commit_message>
<xml_diff>
--- a/measure_point/measure_point.xlsx
+++ b/measure_point/measure_point.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DeepCFD2025\jnjpcode\POD\measure_point\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17DFCFAF-BB20-4971-B811-EC627C2DC1B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C69AE5D5-BCF5-44C3-9C6D-230B6E696921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2660" yWindow="1530" windowWidth="12830" windowHeight="13750" xr2:uid="{B5886C22-FCE1-41C5-937C-84926399ADA4}"/>
+    <workbookView xWindow="8480" yWindow="2510" windowWidth="12830" windowHeight="13750" xr2:uid="{B5886C22-FCE1-41C5-937C-84926399ADA4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>x</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -47,6 +47,10 @@
   </si>
   <si>
     <t>z</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>index</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -431,13 +435,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12FC7FED-4626-41CB-A096-9E550D8DCCC3}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -447,8 +451,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0.21875081597375501</v>
       </c>
@@ -458,8 +465,11 @@
       <c r="C2">
         <v>1.00679451171937</v>
       </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>-0.18128674226397501</v>
       </c>
@@ -469,8 +479,11 @@
       <c r="C3">
         <v>1.00515874149613</v>
       </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>-0.17894598976522999</v>
       </c>
@@ -480,8 +493,11 @@
       <c r="C4">
         <v>1.99789309508946</v>
       </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>0.21827485753806999</v>
       </c>
@@ -491,8 +507,11 @@
       <c r="C5">
         <v>1.99574787257527</v>
       </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>-7.96189829712215E-3</v>
       </c>
@@ -501,6 +520,9 @@
       </c>
       <c r="C6">
         <v>2.03775392154219</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>